<commit_message>
02.01.000 follow-ups: MiniLaser Current Draw Reference (html/xlsx no fills/help), no empty guide on MiniLaser-only sheets, Arrangement 1 carries MiniLasers, class order area→project→SFD, .pl MiniLasers non-pre-engineered by default with override; regression suites in tests/regression
</commit_message>
<xml_diff>
--- a/ModuLaser_Current_Draw_Reference.xlsx
+++ b/ModuLaser_Current_Draw_Reference.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,49 +26,20 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00555555"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00333333"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E4C87"/>
-        <bgColor rgb="002E4C87"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -80,39 +51,28 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00999999"/>
-      </left>
-      <right style="thin">
-        <color rgb="00999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="00999999"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00999999"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -120,95 +80,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>ModuLaser Battery Calculator</author>
-  </authors>
-  <commentList>
-    <comment ref="C5" authorId="0" shapeId="0">
-      <text>
-        <t>Manufacturer worksheet publishes only the LEDS-Off state for Minimum Display (no TFT) at 18V — no LEDS-On figure is available in the source data, so this is the highest published value rather than a true TFT-On/LEDS-On worst case.</t>
-      </text>
-    </comment>
-    <comment ref="C7" authorId="0" shapeId="0">
-      <text>
-        <t>No separate current-draw entry exists for Command Display in the source manufacturer table. This reuses the Standard Display figure, consistent with the calculator's own treatment of both display types as electrically identical (FHSD8310-ULF and FHSD8320-ULF share the same 232 mA rating in the calculator).</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,7 +372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -517,414 +389,639 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>18V figures per manufacturer worksheet; 24V figures as embedded in the ModuLaser Battery Calculator</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Module Type</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>18V Current (mA)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>24V Current (mA) — as used by calculator</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Minimum Display</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>FHSD8300-ULF</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="3" t="n">
         <v>242</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="3" t="n">
         <v>210</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Standard Display</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>FHSD8310-ULF</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="3" t="n">
         <v>266</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="3" t="n">
         <v>232</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Command Display</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>FHSD8320-ULF</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="3" t="n">
         <v>266</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="3" t="n">
         <v>232</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 1)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
         <v>250</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="3" t="n">
         <v>218</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 2)</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
         <v>279</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="3" t="n">
         <v>234</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 3)</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
         <v>305</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="3" t="n">
         <v>255</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 4)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
         <v>330</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="3" t="n">
         <v>279</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 5)</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="n">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
         <v>358</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="3" t="n">
         <v>301</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 6)</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
         <v>380</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="3" t="n">
         <v>330</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 7)</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
         <v>430</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="3" t="n">
         <v>363</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 8)</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
         <v>465</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="3" t="n">
         <v>393</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 9)</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
         <v>517</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="3" t="n">
         <v>431</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 10)</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
         <v>566</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="3" t="n">
         <v>471</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 11)</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
         <v>615</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="3" t="n">
         <v>506</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 12)</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
         <v>685</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="3" t="n">
         <v>552</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 13)</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
         <v>733</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="3" t="n">
         <v>602</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 14)</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
         <v>786</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="3" t="n">
         <v>646</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 15)</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
         <v>872</v>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="3" t="n">
         <v>712</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Detector (Fan Speed 16)</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>FHSD8330-ULF</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8330-ULF</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
         <v>1021</v>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="3" t="n">
         <v>762</v>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>MiniLaser ASD (standalone) — by Fan Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Module Type</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Standby (mA, 24 VDC)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Alarm (mA, 24 VDC) — as used by calculator</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 1)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 2)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 3)</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>157</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 4)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 5)</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 6)</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 7)</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>255</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 8)</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>285</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 9)</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>MiniLaser (Fan Speed 10)</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>FHSD8075-ULF</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>365</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>• 18V figures shown are taken directly from the manufacturer's current-draw worksheet at the 18.0V test point ("New UL Values").</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>• 24V figures are the values embedded in the ModuLaser Battery Calculator, which do not match either the 18.0V or 20.4V rows in the manufacturer worksheet exactly — they reflect a separate reference point used when the calculator was built.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>• Display rows are collapsed to a single current value each, per the calculator's own model (which does not distinguish TFT or LEDS state) — the TFT-On/LEDS-On (highest-draw) state was used to select the corresponding 18V figure. See cell comments on Minimum Display and Command Display for the two cases where that exact combination wasn't available in the source data and a documented substitution was made.</t>
         </is>
       </c>
     </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>• MiniLaser (FHSD8075-ULF): current at 24 VDC from the MiniLaser Installation Manual; alarm draw = fan-speed draw (standby = alarm). No 18V figure is published for the MiniLaser. Each MiniLaser is on its own dedicated AUX circuit (35 mA per-circuit overhead, 3.0 A limit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>• MiniLaser I/O Expansion Module (9-30521) and Expansion Housing (9-30520): no current draw published; treated as no added draw (per Brent, 2026-10-16).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A41:D41"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A42:D42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
02.01.000: arrangement card shown alongside the Disparate-clusters warning (Brent 9:02 PM); flag fires on A/BPS only when clusters share a pathway (QA F8); M p.66 MiniLaser pipe limits enforced (F1); CDR xlsx explicit black font (F6); test hygiene (F3/F4); docs
</commit_message>
<xml_diff>
--- a/ModuLaser_Current_Draw_Reference.xlsx
+++ b/ModuLaser_Current_Draw_Reference.xlsx
@@ -21,16 +21,18 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
   </fonts>

</xml_diff>